<commit_message>
Update 20250411 Ajustes de posición en impresora 3D.xlsx
</commit_message>
<xml_diff>
--- a/Captura de datos medidas cama/20250411 Ajustes de posición en impresora 3D.xlsx
+++ b/Captura de datos medidas cama/20250411 Ajustes de posición en impresora 3D.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="133">
   <si>
     <t>Ancho de la cama en X</t>
   </si>
@@ -388,6 +388,33 @@
   </si>
   <si>
     <t>#   decrementa la distancia.</t>
+  </si>
+  <si>
+    <t>En determinadas circunstancias</t>
+  </si>
+  <si>
+    <t>en las que queremos medir</t>
+  </si>
+  <si>
+    <t>hay maquinas que no son capaces</t>
+  </si>
+  <si>
+    <t xml:space="preserve">de alcanzar las posiciones </t>
+  </si>
+  <si>
+    <t>en este bloque puedes ver si alguna</t>
+  </si>
+  <si>
+    <t>de las posiciones no es alcanzable</t>
+  </si>
+  <si>
+    <t>Chequeo de medidas:</t>
+  </si>
+  <si>
+    <t>Medidas</t>
+  </si>
+  <si>
+    <t>Chequeo</t>
   </si>
 </sst>
 </file>
@@ -421,7 +448,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -443,6 +470,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF00B0F0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -483,7 +516,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -516,11 +549,185 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="23">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
 </styleSheet>
 </file>
@@ -989,7 +1196,7 @@
       </c>
       <c r="H8" s="10">
         <f>IF(B9&gt;0,B7-H31,B7-H31-(0-B9))</f>
-        <v>191.2</v>
+        <v>185.5</v>
       </c>
       <c r="I8" s="10" t="s">
         <v>44</v>
@@ -1004,7 +1211,7 @@
         <v>2</v>
       </c>
       <c r="B9" s="9">
-        <v>-31.8</v>
+        <v>-37.5</v>
       </c>
       <c r="D9" t="s">
         <v>17</v>
@@ -1236,7 +1443,7 @@
       </c>
       <c r="E35" s="10">
         <f>B9</f>
-        <v>-31.8</v>
+        <v>-37.5</v>
       </c>
       <c r="G35" t="s">
         <v>34</v>
@@ -1286,7 +1493,7 @@
       </c>
       <c r="E41" s="10">
         <f>B9</f>
-        <v>-31.8</v>
+        <v>-37.5</v>
       </c>
       <c r="G41" t="s">
         <v>89</v>
@@ -1410,15 +1617,19 @@
         <v>5</v>
       </c>
     </row>
-    <row r="50" spans="4:10" ht="13.5" thickBot="1"/>
+    <row r="50" spans="4:10" ht="13.5" thickBot="1">
+      <c r="E50" s="7" t="s">
+        <v>131</v>
+      </c>
+    </row>
     <row r="51" spans="4:10" ht="13.5" thickBot="1">
       <c r="D51" t="s">
         <v>103</v>
       </c>
-      <c r="E51" s="9">
+      <c r="E51" s="14">
         <v>26.5</v>
       </c>
-      <c r="F51" s="9">
+      <c r="F51" s="14">
         <v>29.5</v>
       </c>
       <c r="G51" t="s">
@@ -1432,10 +1643,10 @@
       <c r="D52" t="s">
         <v>104</v>
       </c>
-      <c r="E52" s="9">
+      <c r="E52" s="14">
         <v>202.5</v>
       </c>
-      <c r="F52" s="9">
+      <c r="F52" s="14">
         <v>29.5</v>
       </c>
       <c r="G52" t="s">
@@ -1449,10 +1660,10 @@
       <c r="D53" t="s">
         <v>105</v>
       </c>
-      <c r="E53" s="9">
+      <c r="E53" s="14">
         <v>202.5</v>
       </c>
-      <c r="F53" s="9">
+      <c r="F53" s="14">
         <v>200.5</v>
       </c>
       <c r="G53" t="s">
@@ -1466,10 +1677,10 @@
       <c r="D54" t="s">
         <v>106</v>
       </c>
-      <c r="E54" s="9">
+      <c r="E54" s="14">
         <v>26.5</v>
       </c>
-      <c r="F54" s="9">
+      <c r="F54" s="14">
         <v>200.5</v>
       </c>
       <c r="G54" t="s">
@@ -1487,71 +1698,121 @@
         <v>111</v>
       </c>
     </row>
-    <row r="56" spans="4:10">
+    <row r="56" spans="4:10" ht="13.5" thickBot="1">
+      <c r="D56" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="E56" s="7" t="s">
+        <v>132</v>
+      </c>
       <c r="G56" t="s">
         <v>91</v>
       </c>
-      <c r="H56" s="10">
+      <c r="H56" s="16">
         <f>E51-$E$41</f>
-        <v>58.3</v>
-      </c>
-      <c r="I56" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="I56" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="J56" s="10">
+      <c r="J56" s="16">
         <f>F51-$E$42</f>
         <v>70</v>
       </c>
     </row>
-    <row r="57" spans="4:10">
+    <row r="57" spans="4:10" ht="13.5" thickBot="1">
+      <c r="D57" t="s">
+        <v>124</v>
+      </c>
+      <c r="E57" s="15" t="str">
+        <f>IF(OR(H56&lt;$E$10,H56&gt;$E$11),"NO VALIDO","CORRECTO")</f>
+        <v>CORRECTO</v>
+      </c>
+      <c r="F57" s="15" t="str">
+        <f>IF(OR(J56&lt;$E$23,J56&gt;$E$24),"NO VALIDO","CORRECTO")</f>
+        <v>CORRECTO</v>
+      </c>
       <c r="G57" t="s">
         <v>92</v>
       </c>
-      <c r="H57" s="10">
+      <c r="H57" s="16">
         <f t="shared" ref="H57:H59" si="2">E52-$E$41</f>
-        <v>234.3</v>
-      </c>
-      <c r="I57" s="10" t="s">
+        <v>240</v>
+      </c>
+      <c r="I57" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="J57" s="10">
+      <c r="J57" s="16">
         <f t="shared" ref="J57:J59" si="3">F52-$E$42</f>
         <v>70</v>
       </c>
     </row>
-    <row r="58" spans="4:10">
+    <row r="58" spans="4:10" ht="13.5" thickBot="1">
+      <c r="D58" t="s">
+        <v>126</v>
+      </c>
+      <c r="E58" s="15" t="str">
+        <f t="shared" ref="E58:E60" si="4">IF(OR(H57&lt;$E$10,H57&gt;$E$11),"NO VALIDO","CORRECTO")</f>
+        <v>CORRECTO</v>
+      </c>
+      <c r="F58" s="15" t="str">
+        <f t="shared" ref="F58:F60" si="5">IF(OR(J57&lt;$E$23,J57&gt;$E$24),"NO VALIDO","CORRECTO")</f>
+        <v>CORRECTO</v>
+      </c>
       <c r="G58" t="s">
         <v>93</v>
       </c>
-      <c r="H58" s="10">
+      <c r="H58" s="16">
         <f t="shared" si="2"/>
-        <v>234.3</v>
-      </c>
-      <c r="I58" s="10" t="s">
+        <v>240</v>
+      </c>
+      <c r="I58" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="J58" s="10">
+      <c r="J58" s="16">
         <f t="shared" si="3"/>
         <v>241</v>
       </c>
     </row>
-    <row r="59" spans="4:10">
+    <row r="59" spans="4:10" ht="13.5" thickBot="1">
+      <c r="D59" t="s">
+        <v>127</v>
+      </c>
+      <c r="E59" s="15" t="str">
+        <f t="shared" si="4"/>
+        <v>CORRECTO</v>
+      </c>
+      <c r="F59" s="15" t="str">
+        <f t="shared" si="5"/>
+        <v>NO VALIDO</v>
+      </c>
       <c r="G59" t="s">
         <v>94</v>
       </c>
-      <c r="H59" s="10">
+      <c r="H59" s="16">
         <f t="shared" si="2"/>
-        <v>58.3</v>
-      </c>
-      <c r="I59" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="I59" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="J59" s="10">
+      <c r="J59" s="16">
         <f t="shared" si="3"/>
         <v>241</v>
       </c>
     </row>
-    <row r="60" spans="4:10">
+    <row r="60" spans="4:10" ht="13.5" thickBot="1">
+      <c r="D60" t="s">
+        <v>125</v>
+      </c>
+      <c r="E60" s="15" t="str">
+        <f t="shared" si="4"/>
+        <v>CORRECTO</v>
+      </c>
+      <c r="F60" s="15" t="str">
+        <f>IF(OR(J59&lt;$E$23,J59&gt;$E$24),"NO VALIDO","CORRECTO")</f>
+        <v>NO VALIDO</v>
+      </c>
       <c r="G60" t="s">
         <v>109</v>
       </c>
@@ -1560,6 +1821,9 @@
       </c>
     </row>
     <row r="61" spans="4:10">
+      <c r="D61" t="s">
+        <v>128</v>
+      </c>
       <c r="G61" t="s">
         <v>107</v>
       </c>
@@ -1568,6 +1832,9 @@
       </c>
     </row>
     <row r="62" spans="4:10">
+      <c r="D62" t="s">
+        <v>129</v>
+      </c>
       <c r="G62" t="s">
         <v>115</v>
       </c>
@@ -1611,6 +1878,34 @@
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="E57:F60">
+    <cfRule type="notContainsText" dxfId="9" priority="9" operator="notContains" text="CORRECTO">
+      <formula>ISERROR(SEARCH("CORRECTO",E57))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="8" priority="10" operator="containsText" text="CORRECTO">
+      <formula>NOT(ISERROR(SEARCH("CORRECTO",E57)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H56:H59">
+    <cfRule type="cellIs" dxfId="7" priority="4" operator="between">
+      <formula>$E$10</formula>
+      <formula>$E$11</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="notBetween">
+      <formula>$E$10</formula>
+      <formula>$E$11</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J56:J59">
+    <cfRule type="cellIs" dxfId="6" priority="2" operator="between">
+      <formula>$E$23</formula>
+      <formula>$E$24</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="5" priority="1" operator="notBetween">
+      <formula>$E$23</formula>
+      <formula>$E$24</formula>
+    </cfRule>
+  </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.11811023622047245" right="0.23622047244094491" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" scale="80" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>

</xml_diff>